<commit_message>
Updated inventory snapshot + dashboard changes
</commit_message>
<xml_diff>
--- a/data/raw/inventory/Week 7/Audio_Array/Inventory Snapshot.xlsx
+++ b/data/raw/inventory/Week 7/Audio_Array/Inventory Snapshot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\inventory\Week 7\Audio_Array\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{579655A5-77F5-401B-99C2-3A3FB093588E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA2FDD3-ED4F-4171-90A6-052F16357F68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D49B0F4C-5F9E-467E-8AD9-9E638F42404F}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$614</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1562,7 +1562,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1572,6 +1572,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1604,7 +1610,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1613,6 +1619,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2114,7 +2123,8 @@
       <c r="D3" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="4">
+        <f>59+72</f>
         <v>131</v>
       </c>
       <c r="J3" s="1" t="s">
@@ -2504,7 +2514,7 @@
       <c r="D18" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="I18" s="1">
+      <c r="I18" s="4">
         <v>105</v>
       </c>
       <c r="J18" s="1" t="s">
@@ -5416,7 +5426,7 @@
       <c r="D130" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="I130" s="1">
+      <c r="I130" s="4">
         <v>30</v>
       </c>
       <c r="J130" s="1" t="s">
@@ -6872,7 +6882,7 @@
       <c r="D186" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="I186" s="1">
+      <c r="I186" s="4">
         <v>0</v>
       </c>
       <c r="J186" s="1" t="s">
@@ -16226,7 +16236,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
+  <autoFilter ref="A1:L614" xr:uid="{76CBFB1B-DC23-4380-8138-4D6BFF18CBC5}"/>
   <conditionalFormatting sqref="A1:B1">
     <cfRule type="duplicateValues" dxfId="6" priority="156"/>
   </conditionalFormatting>

</xml_diff>